<commit_message>
CRM: drop LenderLink (underwriting service) and Arc (spam) per Steve — Harrison-intro pipeline only
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -740,206 +740,73 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>LenderLink</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Marketplace / broker (PH)</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>1. Intro made</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>n/a (marketplace)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Yash Sokhal (Commercial Director)</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>yash@lenderlink.ph</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Inbound outreach, 2026-08-11</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Ces scheduling first meeting (their 9/1 ask); decide if worth a listen</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>PH-based lender marketplace, BGC office. Being handled by Ces (Frances Politud).</t>
-        </is>
-      </c>
-    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Arc (joinarc.com)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Venture-debt marketplace (US)</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>0. Inbound — not engaged</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Pitched ~1/3 of last equity round, 'high single digits'</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Eli Pollak (Capital Markets)</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>eli@goarcfinance.com</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Cold inbound, 2026-09-04</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Decide: respond or ignore (both emails sitting in Gmail spam)</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>YC W22; non-exclusive placement process. Followed up 9/9 unanswered.</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Advisors / Referrers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Intros made</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Last touch</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Advisors / Referrers</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Firm</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Intros made</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Last touch</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Harrison Emmett-Lee</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital (UK)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Capital markets advisor / connector</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>FPF (3/06), Accial (3/06)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Recurring 'Capital Markets Catch up' cadence Mar–Jun 2026; joined early FPF/Accial calls. Clarissa Morrison cc'd on facility threads.</t>
         </is>
@@ -967,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1041,17 +908,17 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>LenderLink</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>In (Yash→Ces)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1061,51 +928,51 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Follow-up asking Ces for meeting times (thread since 8/11).</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04/09</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>In (cold)</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Email (spam folder)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Venture-debt marketplace pitch: ~1/3 of last raise at 'high single digits'; follow-up 9/9. Unanswered.</t>
+          <t>[Content not in local Mail — confirm.] Last message on 'Zed First Facility' thread; ball with Zed?</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-11/13</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>In/Out (Carrie↔Steve)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1115,51 +982,51 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>[Content not in local Mail — confirm.] Post-call exchange after ~8/10 call (Fireflies recording notification on thread).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>[Content not in local Mail — confirm.] Last message on 'Zed First Facility' thread; ball with Zed?</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11/13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>In/Out (Carrie↔Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1169,51 +1036,51 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>[Content not in local Mail — confirm.] Post-call exchange after ~8/10 call (Fireflies recording notification on thread).</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1223,19 +1090,19 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1250,14 +1117,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1267,7 +1134,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1277,24 +1144,24 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1304,140 +1171,86 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out/In</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email + DocuSign</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>FPF + Accial</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Harrison)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>FPF</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Call</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>FPF + Accial</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>In (Harrison)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
CRM: Accial August exchange recovered — stage 3, their typical terms recorded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>2. First call</t>
+          <t>3. NDA / early materials</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -726,21 +726,20 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>[Confirm: content of Carrie's 8/11 &amp; 8/19 emails — call happened ~8/10 (Fireflies recording on thread). Re-engage or park?]</t>
+          <t>BALL WITH ZED since 8/19: review/sign their NDA (fill in Zed details), then open initial data room — their list: corp deck, monthly financials since inception, projections, product description + loan tape with full loan-level history, corp structure, cap table + borrowing list.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Intro stalled twice (Mar, May); revived 6/24. Manila meet missed (Steve paternity leave, Jul). Call ~8/10; last inbound from Carrie 8/19 — thread ends with them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
+          <t>Intro call 8/10 (Fireflies recorded). Their typical structure (Carrie, 8/19): tenor 2–4 yrs (~6-mo drawdown, long interest-only with recycling, amortization matched to asset tenor); fixed commitment with borrowing-base compliance once drawn; prefers SG/global holdco (PH onshore possible); off-balance-sheet SPV + corporate guarantee from holdco; USD. Intro stalled twice (Mar, May); revived 6/24.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
@@ -834,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -955,14 +954,14 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>[Content not in local Mail — confirm.] Last message on 'Zed First Facility' thread; ball with Zed?</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11/13</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -972,7 +971,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>In/Out (Carrie↔Steve)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -982,105 +981,105 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>[Content not in local Mail — confirm.] Post-call exchange after ~8/10 call (Fireflies recording notification on thread).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1090,19 +1089,19 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1117,14 +1116,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1134,7 +1133,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1144,24 +1143,24 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1171,86 +1170,140 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Out/In</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Email + DocuSign</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
Accial NDA redline sent 9/11: CRM updated, NDA files archived to processed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -721,17 +721,17 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH ZED since 8/19: review/sign their NDA (fill in Zed details), then open initial data room — their list: corp deck, monthly financials since inception, projections, product description + loan tape with full loan-level history, corp structure, cap table + borrowing list.</t>
+          <t>BALL WITH ACCIAL: redlined NDA sent 9/11 (survival 3yr + trade secrets; consent-gated third-party sharing; no-contest struck; prompt notice; Zed Financial, Inc. as counterparty). Awaiting their counter/signature, then open initial data room (their 8/11 list).</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -885,12 +885,12 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -900,14 +900,14 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -927,24 +927,24 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -954,14 +954,14 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -981,14 +981,14 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1025,29 +1025,29 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1057,19 +1057,19 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -1079,34 +1079,34 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1116,14 +1116,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1143,19 +1143,19 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1170,24 +1170,24 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1197,14 +1197,14 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1224,41 +1224,41 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -1268,42 +1268,69 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out/In</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email + DocuSign</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
FPF 9/18 catch-up call: Granola notes archived, tracker v20, CRM + README updated (terms or pass expected wk of 9/28)
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -629,7 +629,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>First facility (size TBD)</t>
+          <t>$5M first facility (Steve's target, stated on 9/18 call)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -654,22 +654,22 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>FPF reviews 9/09 response sheet + funds-flow diagram; call offered Tue/Wed 9/15–16; FPF owes indicative terms (committed on 8/12 call)</t>
+          <t>BALL WITH FPF: Raymond takes Zed to an internal meeting wk of 9/21; expects to send indicative terms or a no-go wk of 9/28. Steve to catch up with Raymond wk of 9/28.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>NDA signed Apr 2026 (CA law, ICC arbitration, Miami venue). Full data room + 28 diligence responses delivered. Deepest conversation in pipeline.</t>
+          <t>NDA signed Apr 2026 (CA law, ICC arbitration, Miami venue). Full data room + 28 diligence responses delivered. Deepest conversation in pipeline. 9/18 catch-up call (Steve × Raymond): no new diligence asks; covered book growth, unit economics, burn/runway, Series B timing. Structure: PHP-denominated onshore facility preferred longer-term; near-term likely offshore (e.g. Singapore holdco) — would be FPF's first Singapore facility, Steve offered to be a resource. Zed wants the first facility closed before starting Series B conversations (~end of 2026; target close mid-2027).</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -880,27 +880,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
+          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
         </is>
       </c>
     </row>
@@ -912,12 +912,12 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -927,14 +927,14 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -954,24 +954,24 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -981,14 +981,14 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -1052,29 +1052,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1084,19 +1084,19 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -1106,34 +1106,34 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1143,14 +1143,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -1170,19 +1170,19 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1197,24 +1197,24 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1224,14 +1224,14 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1251,41 +1251,41 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -1295,42 +1295,69 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out/In</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email + DocuSign</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
Accial 10/14 call processed: notes archived, tracker v21 + item 14 (interchange data, Open), CRM to deep diligence, README owes list; 10/01 structure handoff filed
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pipeline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Correspondence Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stage Definitions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondence Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stage Definitions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -659,12 +659,12 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH FPF: Raymond takes Zed to an internal meeting wk of 9/21; expects to send indicative terms or a no-go wk of 9/28. Steve to catch up with Raymond wk of 9/28.</t>
+          <t>BALL WITH FPF: indicative terms or pass still outstanding; per 10/14 Accial call, 'another fund' (presumed FPF) takes Zed to IC Mon 2026-10-19. Chase if nothing by 10/23.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -691,12 +691,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>3. NDA / early materials</t>
+          <t>5. Deep diligence</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>$5M initial, capacity to $10M (Accial min ticket ~$5M; open to tranching e.g. $3M+$2M)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -721,22 +721,22 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH ACCIAL: redlined NDA sent 9/11 (survival 3yr + trade secrets; consent-gated third-party sharing; no-contest struck; prompt notice; Zed Financial, Inc. as counterparty). Awaiting their counter/signature, then open initial data room (their 8/11 list).</t>
+          <t>BALL WITH ACCIAL: propose facility structure (SPV vs holdco/opco loan w/ receivables security at $5M, SPV at scale) + indicative terms after their IC, timed with the other fund's IC (Mon 10/19). Zed owes interchange data (tracker 14). Debrief the 10/16 Manila meeting.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Intro call 8/10 (Fireflies recorded). Their typical structure (Carrie, 8/19): tenor 2–4 yrs (~6-mo drawdown, long interest-only with recycling, amortization matched to asset tenor); fixed commitment with borrowing-base compliance once drawn; prefers SG/global holdco (PH onshore possible); off-balance-sheet SPV + corporate guarantee from holdco; USD. Intro stalled twice (Mar, May); revived 6/24.</t>
+          <t>Intro call 8/10 (Fireflies recorded). Their typical structure (Carrie, 8/19): tenor 2–4 yrs (~6-mo drawdown, long interest-only with recycling, amortization matched to asset tenor); fixed commitment with borrowing-base compliance once drawn; prefers SG/global holdco (PH onshore possible); off-balance-sheet SPV + corporate guarantee from holdco; USD. Intro stalled twice (Mar, May); revived 6/24. NDA executed and data room opened between 9/11 and 10/14 [dates to confirm]; Mikko (risk) reviewed data room. 10/14 diligence call: no financial concerns given equity raised; focus on portfolio track record/economics. Accial view on structure: has done SPVs mostly at $10M+; sub-$10M usually loan to holdco/opco secured on receivables, SPV at scale; US-based fund with US-law capability → US-domiciled SPV feasible. 10/16 Manila in-person: Lawrence (CIO) + Mikko × John (CCO) + Aubrey (Head of Finance).</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -880,12 +880,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -900,14 +900,14 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
+          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -917,24 +917,24 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie)</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>In person, Manila</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
+          <t>Lawrence (CIO) + Mikko (risk) × John (CCO) + Aubrey (Head of Finance). Scheduled per the 10/14 call; outcome not yet recorded.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -944,34 +944,34 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -981,24 +981,24 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1008,24 +1008,24 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -1062,14 +1062,14 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -1079,115 +1079,115 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1224,14 +1224,14 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1251,24 +1251,24 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1278,86 +1278,140 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Out/In</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Email + DocuSign</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
CRM: Accial 10/16 outcome, contacts, 10/13 internal-share row, log re-sorted; METHODS entry for the Manila debrief
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Febe Rahellea (VP of Investment); Lawrence Chua; Carrie Ruh</t>
+          <t>Febe Rahellea (VP Investment); Lawrence Chua (CIO); Carrie Ruh; Mikko (risk analyst); Marco (ex-Zed Partnerships Lead candidate, chose Accial)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH ACCIAL: propose facility structure (SPV vs holdco/opco loan w/ receivables security at $5M, SPV at scale) + indicative terms after their IC, timed with the other fund's IC (Mon 10/19). Zed owes interchange data (tracker 14). Debrief the 10/16 Manila meeting.</t>
+          <t>BALL WITH BOTH: Zed owes interchange data (tracker 14) + breakeven-scale answer (tracker 15) — send week of 10/19. Accial owes structure proposal (SPV vs direct receivables-secured loan; US SPV feasibility) + feedback/IOI, targeting before year-end.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Intro call 8/10 (Fireflies recorded). Their typical structure (Carrie, 8/19): tenor 2–4 yrs (~6-mo drawdown, long interest-only with recycling, amortization matched to asset tenor); fixed commitment with borrowing-base compliance once drawn; prefers SG/global holdco (PH onshore possible); off-balance-sheet SPV + corporate guarantee from holdco; USD. Intro stalled twice (Mar, May); revived 6/24. NDA executed and data room opened between 9/11 and 10/14 [dates to confirm]; Mikko (risk) reviewed data room. 10/14 diligence call: no financial concerns given equity raised; focus on portfolio track record/economics. Accial view on structure: has done SPVs mostly at $10M+; sub-$10M usually loan to holdco/opco secured on receivables, SPV at scale; US-based fund with US-law capability → US-domiciled SPV feasible. 10/16 Manila in-person: Lawrence (CIO) + Mikko × John (CCO) + Aubrey (Head of Finance).</t>
+          <t>Intro call 8/10 (Fireflies recorded). Their typical structure (Carrie, 8/19): tenor 2–4 yrs (~6-mo drawdown, long interest-only with recycling, amortization matched to asset tenor); fixed commitment with borrowing-base compliance once drawn; prefers SG/global holdco (PH onshore possible); off-balance-sheet SPV + corporate guarantee from holdco; USD. Intro stalled twice (Mar, May); revived 6/24. NDA executed and data room opened between 9/11 and 10/14 [dates to confirm]; Mikko (risk) reviewed data room. 10/14 diligence call: no financial concerns given equity raised; focus on portfolio track record/economics. Accial view on structure: has done SPVs mostly at $10M+; sub-$10M usually loan to holdco/opco secured on receivables, SPV at scale; US-based fund with US-law capability → US-domiciled SPV feasible. 10/16 Manila in-person: Lawrence (CIO) + Mikko × John (CCO) + Aubrey (Head of Finance). 10/16 Manila in-person (Lawrence, Mikko, Marco × Jon, Auvrey) went well; questions matched prep; one unanticipated: breakeven scale. Marco will nudge internally; concern = unit economics / annualized yield. Verbal disclosures incl. installment eligibility rules, 16K cardholders / $30M originated, model V1→V2.</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -880,7 +880,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
@@ -890,24 +890,24 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Video call (Granola notes)</t>
+          <t>In person, Manila</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
+          <t>Lawrence (CIO) + Mikko (risk) + Marco × Jon (CCO) + Auvrey (Head of Finance); Steve absent. Went well per Auvrey; questions as prepared. Unanticipated: breakeven scale — Zed to revert (tracker 15). Also asked: growth plans post-debt (product-led), other demographics (no — young professionals). Marco: will nudge internally; concern is unit economics / annualized yield.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -917,71 +917,71 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>In person, Manila</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lawrence (CIO) + Mikko (risk) × John (CCO) + Aubrey (Head of Finance). Scheduled per the 10/14 call; outcome not yet recorded.</t>
+          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Video call (Granola notes)</t>
+          <t>Slack #accial-ph-visit</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
+          <t>Steve shared the facility-structure note (v6) with the Zed team as a Google Doc copy ahead of the Manila visit; Auvrey posted Notion notes of the 10/14 call. Internal only — nothing sent to Accial.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
+          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1035,24 +1035,24 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1062,14 +1062,14 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1089,14 +1089,14 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1116,14 +1116,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1133,29 +1133,29 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1165,19 +1165,19 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -1187,34 +1187,34 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1224,14 +1224,14 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -1251,19 +1251,19 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1278,24 +1278,24 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1305,14 +1305,14 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1332,41 +1332,41 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -1376,42 +1376,69 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out/In</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email + DocuSign</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
Revert Excel re-saves swept into 7da2135 (tapes restored to Box-identical, sent 9/09 sheet restored); CRM: log 10/16 Accial email + next action; METHODS note
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH BOTH: Zed owes interchange data (tracker 14) + breakeven-scale answer (tracker 15) — send week of 10/19. Accial owes structure proposal (SPV vs direct receivables-secured loan; US SPV feasibility) + feedback/IOI, targeting before year-end.</t>
+          <t>BALL WITH ZED: send interchange data (tracker 14) + breakeven answer (tracker 15) with a timing ask; Steve's 10/16 thank-you/offer email unanswered as of 10/26. Then Accial owes structure proposal + IOI (targeting before year-end).</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -890,24 +890,24 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Out (Steve→Carrie, cc Lawrence/Mikko/team)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>In person, Manila</t>
+          <t>Email (thread 'Zed First Facility')</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Lawrence (CIO) + Mikko (risk) + Marco × Jon (CCO) + Auvrey (Head of Finance); Steve absent. Went well per Auvrey; questions as prepared. Unanticipated: breakeven scale — Zed to revert (tracker 15). Also asked: growth plans post-debt (product-led), other demographics (no — young professionals). Marco: will nudge internally; concern is unit economics / annualized yield.</t>
+          <t>Thank-you after the Manila visit; offered a call with Danielle on marketing strategy, product roadmap and post-debt plans. Sent Fri 3:58 PM PT = Sat AM Manila. No reply as of 10/26. Did not include the two owed items (interchange data, breakeven answer).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -917,24 +917,24 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Video call (Granola notes)</t>
+          <t>In person, Manila</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
+          <t>Lawrence (CIO) + Mikko (risk) + Marco × Jon (CCO) + Auvrey (Head of Finance); Steve absent. Went well per Auvrey; questions as prepared. Unanticipated: breakeven scale — Zed to revert (tracker 15). Also asked: growth plans post-debt (product-led), other demographics (no — young professionals). Marco: will nudge internally; concern is unit economics / annualized yield.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -944,71 +944,71 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Slack #accial-ph-visit</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Steve shared the facility-structure note (v6) with the Zed team as a Google Doc copy ahead of the Manila visit; Auvrey posted Notion notes of the 10/14 call. Internal only — nothing sent to Accial.</t>
+          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Video call (Granola notes)</t>
+          <t>Slack #accial-ph-visit</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
+          <t>Steve shared the facility-structure note (v6) with the Zed team as a Google Doc copy ahead of the Manila visit; Auvrey posted Notion notes of the 10/14 call. Internal only — nothing sent to Accial.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
+          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
         </is>
       </c>
     </row>
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1062,24 +1062,24 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1089,14 +1089,14 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1116,14 +1116,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1143,14 +1143,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -1160,29 +1160,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1192,19 +1192,19 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -1214,34 +1214,34 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -1278,19 +1278,19 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1305,24 +1305,24 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1332,14 +1332,14 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1359,41 +1359,41 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -1403,42 +1403,69 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out/In</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email + DocuSign</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>

<commit_message>
CRM: 10/28 yield-analysis sends to Accial and FPF; Carrie role; next steps
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Debt Fundraising CRM.xlsx
+++ b/Analyses (internal)/Debt Fundraising CRM.xlsx
@@ -654,17 +654,17 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH FPF: indicative terms or pass still outstanding; per 10/14 Accial call, 'another fund' (presumed FPF) takes Zed to IC Mon 2026-10-19. Chase if nothing by 10/23.</t>
+          <t>BALL WITH FPF: indicative terms or pass (outstanding since 9/18); yield analysis sent 10/28 as a nudge.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-11-04</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Febe Rahellea (VP Investment); Lawrence Chua (CIO); Carrie Ruh; Mikko (risk analyst); Marco (ex-Zed Partnerships Lead candidate, chose Accial)</t>
+          <t>Febe Rahellea (VP Investment); Lawrence Chua (CIO); Carrie Ruh; Mikko (risk analyst); Marco (ex-Zed Partnerships Lead candidate, chose Accial) — Carrie Ruh: junior principal, not on the IC (Steve 10/28); Lawrence Chua (CIO) and Mikko Vitug (risk) are the evaluators; Marco Gancayco (joined Manila)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -721,17 +721,17 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>BALL WITH ZED: send the breakeven answer promised in Manila (tracker 15) with a timing ask; optionally attach the interchange table Steve offered on the 10/14 call (tracker 14 — offered, not requested). Steve's 10/16 thank-you email unanswered as of 10/26. Then Accial owes structure proposal + IOI (targeting before year-end).</t>
+          <t>BALL WITH ACCIAL: structure proposal + feedback/IOI (targeting before year-end). Zed: Box upload of the yield analysis; breakeven answer (item 15) still owed.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -880,7 +880,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
@@ -890,51 +890,51 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie, cc Lawrence/Mikko/team)</t>
+          <t>Out (Steve→Carrie, Lawrence, Mikko; cc Jon/Auvrey/Danielle; Marco not on thread)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Email (thread 'Zed First Facility')</t>
+          <t>Email (thread 'Zed First Facility'), 7:54 PM PT</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Thank-you after the Manila visit; offered a call with Danielle on marketing strategy, product roadmap and post-debt plans. Sent Fri 3:58 PM PT = Sat AM Manila. No reply as of 10/26. Did not include the two owed items (interchange data, breakeven answer).</t>
+          <t>Sent 'Zed Portfolio Yield Analysis.xlsx' (tracker 16): gross/net yield on receivables by book month, Jun–Aug 2026; framed as 'for the funds we're in diligence with'; said the file will also go into the data room (Box upload pending). Loss basis ≥90 DPD ex-FPD 1.15%; net yield 24.0%.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>In person, Manila</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lawrence (CIO) + Mikko (risk) + Marco × Jon (CCO) + Auvrey (Head of Finance); Steve absent. Went well per Auvrey; questions as prepared. Unanticipated: breakeven scale — Zed to revert (tracker 15). Also asked: growth plans post-debt (product-led), other demographics (no — young professionals). Marco: will nudge internally; concern is unit economics / annualized yield.</t>
+          <t>Sent the same 'Zed Portfolio Yield Analysis.xlsx'; pointed Raymond to the Loss Rate tab for 2026 vintages (his 8/26 ask, item 13.1): May and June vintages 0.91% / 0.34%. First FPF-facing artifact since the 9/09 responses; indicative terms still outstanding.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -944,24 +944,24 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out (Steve→Carrie, cc Lawrence/Mikko/team)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Video call (Granola notes)</t>
+          <t>Email (thread 'Zed First Facility')</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
+          <t>Thank-you after the Manila visit; offered a call with Danielle on marketing strategy, product roadmap and post-debt plans. Sent Fri 3:58 PM PT = Sat AM Manila. No reply as of 10/26. Did not include the two owed items (interchange data, breakeven answer).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -971,29 +971,29 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Slack #accial-ph-visit</t>
+          <t>In person, Manila</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Steve shared the facility-structure note (v6) with the Zed team as a Google Doc copy ahead of the Manila visit; Auvrey posted Notion notes of the 10/14 call. Internal only — nothing sent to Accial.</t>
+          <t>Lawrence (CIO) + Mikko (risk) + Marco × Jon (CCO) + Auvrey (Head of Finance); Steve absent. Went well per Auvrey; questions as prepared. Unanticipated: breakeven scale — Zed to revert (tracker 15). Also asked: growth plans post-debt (product-led), other demographics (no — young professionals). Marco: will nudge internally; concern is unit economics / annualized yield.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
+          <t>Diligence call, Steve × Carrie + Mikko. Accial had reviewed the data room; no financial concerns; focus on portfolio economics. Steve walked through three revenue streams, ~1.6% interchange, 1.87% lifetime loss, 33.9% revolvers, write-offs from Q4. Structure: both sides prefer SPV but at $5M likely holdco/opco loan secured on receivables with SPV at scale; US SPV feasible for Accial. Actions: Zed → interchange data; Accial → structure proposal + indicative terms after IC.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1025,24 +1025,24 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Carrie)</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Slack #accial-ph-visit</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
+          <t>Steve shared the facility-structure note (v6) with the Zed team as a Google Doc copy ahead of the Manila visit; Auvrey posted Notion notes of the 10/14 call. Internal only — nothing sent to Accial.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -1052,34 +1052,34 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve→Raymond)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Video call (Granola notes)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
+          <t>Catch-up after the 9/11 response sheet, Steve × Raymond. No new diligence questions. Steve walked through book growth (~$4M), unit economics, burn/runway and Series B timing; stated $5M target facility, PHP onshore preference with offshore/Singapore holdco as the likely near-term structure. Raymond: internal FPF meeting wk of 9/21, indicative terms or no-go wk of 9/28; catch-up planned that week.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>In (Raymond)</t>
+          <t>Out (Steve→Carrie)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1089,24 +1089,24 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
+          <t>Sent redlined NDA (tracked changes): 3-yr survival + trade-secret carve-out, third-party sharing consent-gated and limited to financing parties excl. competitors, no-contest sentence struck, prompt compelled-disclosure notice, entity filled as Zed Financial, Inc. (DE).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>In (Carrie)</t>
+          <t>Out (Steve→Raymond)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1116,24 +1116,24 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
+          <t>Sent Diligence Responses_20260909.xlsx (initial + 8/26 follow-up tabs); confirmed Box 'Product' folder with funds-flow diagram; offered call Tue/Wed 9/15–16.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>In (Raymond)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1143,14 +1143,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
+          <t>8 follow-up diligence questions (tracker items 6–13); asked for call times.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -1170,14 +1170,14 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
+          <t>Answered Steve's structuring questions inline: tenor 2–4 yrs (6-mo drawdown, IO w/ recycling, asset-matched amortization); fixed commitment + borrowing base once drawn; SG/global holdco preferred; off-BS SPV with holdco corporate guarantee; USD. Awaiting Zed's NDA comments/signature.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -1187,115 +1187,115 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Zoom (Fireflies recorded)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
+          <t>Will review NDA; asked how Accial thinks about tenor, sizing (borrowing base vs fixed), domicile (on/offshore), SPV/recourse/warrants, USD vs PHP.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Carrie)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
+          <t>Post-call follow-up: NDA template sent; initial data-room request list (corp deck, monthly financials since inception, projections, product description + full loan-level tape, corp structure, cap table + borrowing list).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Out (Josif)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom (Fireflies recorded)</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
+          <t>Intro call — Steve × Carrie/Febe/Lawrence; structuring not covered in detail (picked up over email).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Zoom</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
+          <t>5.1-scope call: transaction-level data not needed; ~2% loss basis discussed; FPF committed to indicative terms after data review.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Out (Steve)</t>
+          <t>Out (Josif)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1305,19 +1305,19 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
+          <t>First response sheet (14 items) + unit economics + revised statement tape.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1332,14 +1332,14 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
+          <t>Bump: 'let me know if you're free to connect in the coming weeks.'</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>In (Febe)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1359,24 +1359,24 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
+          <t>Missed Manila 7/29–31 window (paternity leave); asked to meet next PH trip.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24/25</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Accial</t>
+          <t>FPF</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>In (Harrison→Febe→Steve)</t>
+          <t>Out (Steve)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1386,86 +1386,140 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
+          <t>Data room link (deck, financials, loan tape, payment tape incl. revolving launch data).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Out/In</t>
+          <t>In (Febe)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Email + DocuSign</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+          <t>Accial team in Manila 7/29–31; proposed in-person meeting.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-06-24/25</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>FPF</t>
+          <t>Accial</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>In (Harrison→Febe→Steve)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Zoom</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+          <t>Thread revived: Febe (now VP) + Lawrence Chua + Carrie Ruh added; intro call proposed for week of 7/06.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Out/In</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Email + DocuSign</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>NDA executed (CA law, ICC arbitration, Miami venue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>FPF</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>First call, Steve × Raymond (scheduled 3/10–3/13 exchange).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>FPF + Accial</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>In (Harrison)</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Tomorrow Capital double intro: Raymond Katz (FPF) and Febe Rahellea (Accial), both 'Zed &amp; …' threads.</t>
         </is>

</xml_diff>